<commit_message>
new pcb power dsitrubution board (balloon)
</commit_message>
<xml_diff>
--- a/POWER_DISTRIBUTION/SOLAR CHARGER/production/SOLAR CHARGER BOM TRACKER.xlsx
+++ b/POWER_DISTRIBUTION/SOLAR CHARGER/production/SOLAR CHARGER BOM TRACKER.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KiCad\PROJECT_SIGMA\STATE ESTIMATION\POWER_DISTRIBUTION\POWER_DISTRIBUTION\SOLAR CHARGER\production\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KiCad\PROJECT_SIGMA\STATE ESTIMATION\POWER_DISTRIBUTION\power_stuff\POWER_DISTRIBUTION\SOLAR CHARGER\production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEB2F1B2-2C71-4E24-9968-FC79A793F4CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16DA0E9C-EFE9-4B55-BF0B-2679FD8FDD18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{87117B3A-459A-4795-82D3-4BBB1E3CEFF8}"/>
+    <workbookView xWindow="7710" yWindow="4545" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{87117B3A-459A-4795-82D3-4BBB1E3CEFF8}"/>
   </bookViews>
   <sheets>
     <sheet name="SOLAR CHARGER_BOM" sheetId="2" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="350">
   <si>
     <t>Reference</t>
   </si>
@@ -1094,6 +1094,15 @@
   </si>
   <si>
     <t>SOLAR CHARGER</t>
+  </si>
+  <si>
+    <t>Need</t>
+  </si>
+  <si>
+    <t>4uF 0805</t>
+  </si>
+  <si>
+    <t>R5 and R6 take from BB</t>
   </si>
 </sst>
 </file>
@@ -1159,13 +1168,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2599,7 +2607,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93E08409-E3EC-43F4-A25C-A48CA95F9ABB}">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="37.140625" customWidth="1"/>
@@ -3096,6 +3104,19 @@
       </c>
       <c r="M14" t="s">
         <v>143</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>347</v>
+      </c>
+      <c r="C16" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -4131,7 +4152,7 @@
       <c r="I2" t="s">
         <v>308</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="N2" t="s">
         <v>309</v>
       </c>
     </row>
@@ -4357,7 +4378,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="5" t="s">
         <v>346</v>
       </c>
     </row>
@@ -4515,7 +4536,7 @@
       </c>
     </row>
     <row r="30" spans="1:6" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="5" t="s">
         <v>345</v>
       </c>
     </row>

</xml_diff>